<commit_message>
feat(local-llm-experiment): 검색전용 지표(Hit@K/MRR/evidence_coverage) 추출 - 재검색 불필요
run_local_model_combo.py가 이미 매 케이스에 저장해두고 있던 hit_at_1/3/5,
reciprocal_rank, evidence_coverage를 metrics 리스트에서 추출(raw 필드만 보느라
놓쳤던 값). 핵심 발견: hit@1/MRR은 작은 청크가 유리, evidence_coverage는 큰 청크가
유리 - 방향이 반대. RAGAS 생성 지표는 evidence_coverage 경향을 따라감.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ragas_eval_data_2026-07-23/deep_chunk_eda_2026-07-25.xlsx
+++ b/docs/ragas_eval_data_2026-07-23/deep_chunk_eda_2026-07-25.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="split_vs_unsplit" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="문서별_chars_per_token" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검색된청크_근사분포(gold129)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="검색전용지표(Hit@K_MRR_evidence)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,13 +29,27 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -49,8 +64,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -23810,4 +23831,484 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>실제 129건 실행에서 기록된 순수 검색(retrieval-only) 지표 - 생성/채점 LLM과 무관, vector_search 결과의 gold 문서 순위만으로 계산됨. 핵심: hit@1/MRR은 작은 청크가 유리, evidence_coverage는 큰 청크가 유리 - 방향이 반대. RAGAS 생성 지표(faithfulness 등)는 evidence_coverage 쪽 경향을 따라감.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>hit_at_1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>hit_at_3</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>hit_at_5</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>reciprocal_rank</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>evidence_coverage</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>tok150</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>129</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.403</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.437</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>tok250</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>129</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.589</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.482</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.527</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>tok512</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>129</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.581</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.445</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.589</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>tok900</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>129</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.326</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.5580000000000001</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.437</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>tok1000</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>129</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.341</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.447</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.698</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>tok1024</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>129</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.341</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0.452</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.729</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>tok1200</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>129</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.372</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.467</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.705</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>tok1500</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>129</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.326</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.443</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.744</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>tok2048</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>129</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.543</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.432</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.744</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>cs300_ov0</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>129</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.388</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.612</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.505</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.497</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>cs600_ov0</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>129</v>
+      </c>
+      <c r="C14" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.535</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.628</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.544</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>cs900_ov0</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>129</v>
+      </c>
+      <c r="C15" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.589</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.451</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.635</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cs1200_ov0</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>129</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0.326</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0.5580000000000001</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0.636</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.701</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>cs1500_ov0</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>129</v>
+      </c>
+      <c r="C17" t="n">
+        <v>0.372</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.589</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0.651</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.474</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.716</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C4:C17">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4:D17">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E4:E17">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F4:F17">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:G17">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00F8696B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="0063BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>